<commit_message>
Auto: Week 33/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W33_2026.xlsx
+++ b/Gulf_Dashboard_W33_2026.xlsx
@@ -695,23 +695,37 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>PRJ-006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SSE</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>[PVfarm(GUE)] Continue Lighting system installation
+[PVfarm(GUE)] Continue Close punch list.
+[PVfarm(GUE)] Continue install Boundary CCTV Pole.
+[PVfarm(GUE)] Installation Pump and Pipe water tank
+[PVfarm(GUE)] Continue Drainage system work
+[PVfarm(GUE)] Continue Grass cutting PV Farm.
+[PVfarm(GUE)] Continue Cleaning PV modules
+[PVfarm(GUE)] Continue Concrete pouring pavement at BESS area
+[PVfarm(GUE)] Thermoscan at equipment.
+[PVfarm(GUE)] Sound test at equipment.
+[115kVSubstation(SIEMENS)] Continue close punch MCC.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -897,232 +911,335 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>PRJ-013</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>GCE</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>The water pressure from the Hi-Tech system (1.5 bar) is insufficient for filling the ser vice water tank.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>PRJ-014</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>GSE</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Detail and spec of equipment at riser pole for PEA approval.
+Detail drawing of water pond.
+Detail drawing of foundation and architecture of BOP building
+Detail of underground pipe of toilet at steam turbine building.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Pouring concrete from EL.+5.45 to El.+8.00
+Boiler : Install water bune
+FGT area: Install bag filter and reactor tower shell.
+STG :Pouring concrete for column, beam and slab for 2nd floor</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>PRJ-015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>KKE</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Bunker building: Concrete pouring for Lift 4 Wall EL +8.00 to +12.45 m. (25 Aug 2026)
+Tipping hall: Completion of concrete pouring for ground slab
+Boiler Erection: Completion of water wall by (30 Aug 26)
+FGT: Completionof installation Spray Reaction tower by 4 Sep 26 and Bag filer house by (1 Sep 26)
+STG &amp; ECB: Completion of concrete pouring for column (EL -0.7 to +3.75 m.) 27 column (28 Aug 26) Completion of Concrete flat slab (EL +0.25 m.) (7 Sep 26)
+BOP: Completion of ground slab for fire water pump shelter (28 Aug 26)
+Manhole and duct bank: Completion of Manhole for priority 1 (30 Sep 26)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>PRJ-016</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>MKP</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;E manpower and subcontractor mobilization in accordance with the working plan and readiness of work permits.
+Detail drawing of fire fighting system for material purchasing.
+Pipe support standard detail drawing for fabrication and procurement of spring pipe supports, which are long-lead items.
+Diesel oil tank drawing: Clarify the drainage arrangement for the diesel oil tank: bottom drain or draw-off sump in accordance with API 650</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Bunker wall concrete pouring at EL +12m.
+Water wall installation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>PRJ-017</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>MPE</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>The BOP workers is insufficient for the workload</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>PRJ-018</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>PFP</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>The BOP workers is insufficient for the workload</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>PRJ-019</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PKP</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Bunker Building: Pouring concrete Lift 2 EL (+1 to +5.45) (Targeted date 6 Sep 26)
+Boiler Island:Pouring concrete slab , Pouring Concrete Reuse water pool
+FGT : Pouring concrete for ground beam , Pouring concrete footing
+STG &amp; ECB: Pouring concrete ground beam +0.25, Pouring concrete Miscellaneous Foundation
+Boiler &amp; Incinerator: Incinerator grate Installation ; Targeted date 4 Sep 26</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>PRJ-020</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>PSD</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Bunker Building: Install Formwork +1.00 to +2.00,Pouring Concrete +1.00 to +2.00 ; Target date 31 Aug 26,Backfill to -2.00 ; Target date 27 Aug 26
+Boiler Island:Backfill before slab work on ground (Z1-Z6),Pouring concrete Reuse water pool
+FGT : Backfill for hand over to mechanical work
+STG &amp; ECB: Pouring concrete column +3.7 ; Target Date 26 Aug 26
+Boiler &amp; Incinerator: Completion of Boiler Drum Installation. ; Targeted date 25 Aug 26
+BOP : Cooling Tower Foundation work ; Targeted date 28 Aug 26 : Demin water Treatment Foundation work : Service Water Tank Foundation work</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>PRJ-021</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>PWW1</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Work Foundation at Bunker to 18.00 m
+Work Foundation at Boiler, FGT, STG area</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>PRJ-022</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>PWW2</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Contractor for Retaining wall south side</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1. Work Foundation at Bunker to 18.00 m
+Work Foundation at Boiler, FGT, STG area</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>PRJ-023</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>TPP</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;E manpower and subcontractor mobilization in accordance with the working plan and readiness of work permits.
+Detail drawing of fire fighting system for material purchasing.
+Pipe support standard detail drawing for fabrication and procurement of spring pipe supports, which are long-lead items.
+Diesel oil tank drawing: Clarify the drainage arrangement for the diesel oil tank: bottom drain or draw-off sump in accordance with API 650.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Bunker wall concrete pouring at EL +16.9m. 2. Water Wall installation</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>PRJ-024</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>TSE</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Detail and spec of equipment at riser pole for PEA approval.
+Detail drawing of water pond.
+Detail drawing of foundation and architecture of BOP building . Detail of underground pipe of toilet at steam turbine building.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Pouring concrete by slip from method From EL.+8.0 to +18.30 m.
+Boiler: Install boiler wall.
+FGT: Install reactor tower and structure.
+STG : Column for second floor at EL +3.70 m</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">

</xml_diff>